<commit_message>
add the final pcb update the bom with lesspriced lidar add the new model of the 3d robot design
</commit_message>
<xml_diff>
--- a/robot-piece-need/BOM.xlsx
+++ b/robot-piece-need/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ysxay\Documents\1st-robot\3D-model\my-first-hardware-robot-yaya\robot-piece-need\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09AF36E1-454D-48D5-9F66-D825701345E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9103658-609C-45B7-9BE9-331CBE17C189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{7C436766-8AF3-42AE-BA18-92A5E0128A52}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10890" xr2:uid="{7C436766-8AF3-42AE-BA18-92A5E0128A52}"/>
   </bookViews>
   <sheets>
     <sheet name="inventaire_robot_clean" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="119">
   <si>
     <t xml:space="preserve">use                        </t>
   </si>
@@ -151,9 +151,6 @@
     <t xml:space="preserve">lidar 360deg                                   </t>
   </si>
   <si>
-    <t>https://www.gotronic.fr/art-capteur-de-distance-rplidar-a1m8-29031.htm</t>
-  </si>
-  <si>
     <t xml:space="preserve">multiplexer to make easier </t>
   </si>
   <si>
@@ -361,20 +358,32 @@
     <t xml:space="preserve">without funding                                </t>
   </si>
   <si>
-    <t>847.4</t>
-  </si>
-  <si>
     <t xml:space="preserve">with funding                                   </t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>https://fr.aliexpress.com/item/1005010536118026.html?spm=a2g0o.productlist.main.16.4e29550dt3ooVQ&amp;algo_pvid=95d3cccf-ca3c-4b92-b2ce-0ef6c6c9a087&amp;algo_exp_id=95d3cccf-ca3c-4b92-b2ce-0ef6c6c9a087-13&amp;pdp_ext_f=%7B%22order%22%3A%225%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2136.19%2136.19%21%21%21265.13%21265.13%21%4021038db317923271695403921e0efa%2112000052737788669%21sea%21FR%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab75b5c11%3Bm03_new_user%3A-29895&amp;curPageLogUid=LApEO82APory&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010536118026%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>wire connection for lidar</t>
+  </si>
+  <si>
+    <t>bcs lidar not with no wire</t>
+  </si>
+  <si>
+    <t>https://shorturl.at/1T9hr</t>
+  </si>
+  <si>
+    <t>767.4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,6 +518,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -807,7 +824,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -850,11 +867,16 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20 % - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20 % - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -884,6 +906,7 @@
     <cellStyle name="Cellule liée" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Entrée" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Insatisfaisant" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Lien hypertexte" xfId="42" builtinId="8"/>
     <cellStyle name="Neutre" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
@@ -1228,8 +1251,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8373D902-D770-4716-8855-EC0D3903F8A2}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.90625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -1277,7 +1303,7 @@
       <c r="C4">
         <v>292</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1291,7 +1317,7 @@
       <c r="C5">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1338,7 +1364,7 @@
       <c r="C9">
         <v>17</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1410,7 +1436,7 @@
       <c r="C15">
         <v>56</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1424,7 +1450,7 @@
       <c r="C16">
         <v>12</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="1" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1438,7 +1464,7 @@
       <c r="C17">
         <v>5</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1452,7 +1478,7 @@
       <c r="C18">
         <v>10</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1488,7 +1514,7 @@
       <c r="C21">
         <v>32</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="1" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1500,94 +1526,94 @@
         <v>42</v>
       </c>
       <c r="C22">
-        <v>120</v>
+        <v>36</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" t="s">
         <v>44</v>
-      </c>
-      <c r="B23" t="s">
-        <v>45</v>
       </c>
       <c r="C23">
         <v>6</v>
       </c>
-      <c r="D23" t="s">
-        <v>46</v>
+      <c r="D23" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
         <v>47</v>
-      </c>
-      <c r="B24" t="s">
-        <v>48</v>
       </c>
       <c r="C24">
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
         <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>51</v>
       </c>
       <c r="C25">
         <v>35</v>
       </c>
-      <c r="D25" t="s">
-        <v>52</v>
+      <c r="D25" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" t="s">
         <v>53</v>
-      </c>
-      <c r="B26" t="s">
-        <v>54</v>
       </c>
       <c r="C26">
         <v>9</v>
       </c>
-      <c r="D26" t="s">
-        <v>55</v>
+      <c r="D26" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" t="s">
         <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>57</v>
       </c>
       <c r="C27">
         <v>9</v>
       </c>
-      <c r="D27" t="s">
-        <v>58</v>
+      <c r="D27" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" t="s">
         <v>59</v>
-      </c>
-      <c r="B28" t="s">
-        <v>60</v>
       </c>
       <c r="C28">
         <v>9</v>
       </c>
       <c r="D28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
@@ -1598,93 +1624,93 @@
         <v>5</v>
       </c>
       <c r="C29">
-        <v>227</v>
+        <v>143</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" t="s">
         <v>64</v>
-      </c>
-      <c r="B31" t="s">
-        <v>65</v>
       </c>
       <c r="C31">
         <v>16</v>
       </c>
-      <c r="D31" t="s">
-        <v>66</v>
+      <c r="D31" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
+        <v>66</v>
+      </c>
+      <c r="B32" t="s">
         <v>67</v>
-      </c>
-      <c r="B32" t="s">
-        <v>68</v>
       </c>
       <c r="C32">
         <v>17</v>
       </c>
       <c r="D32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" t="s">
         <v>70</v>
-      </c>
-      <c r="B33" t="s">
-        <v>71</v>
       </c>
       <c r="C33">
         <v>17</v>
       </c>
-      <c r="D33" t="s">
-        <v>72</v>
+      <c r="D33" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" t="s">
         <v>73</v>
-      </c>
-      <c r="B34" t="s">
-        <v>74</v>
       </c>
       <c r="C34">
         <v>17</v>
       </c>
-      <c r="D34" t="s">
-        <v>75</v>
+      <c r="D34" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
+        <v>75</v>
+      </c>
+      <c r="B35" t="s">
         <v>76</v>
-      </c>
-      <c r="B35" t="s">
-        <v>77</v>
       </c>
       <c r="C35">
         <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" t="s">
         <v>5</v>
@@ -1693,207 +1719,239 @@
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" t="s">
         <v>81</v>
-      </c>
-      <c r="B37" t="s">
-        <v>82</v>
       </c>
       <c r="C37">
         <v>9</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B38" t="s">
         <v>84</v>
-      </c>
-      <c r="B38" t="s">
-        <v>85</v>
       </c>
       <c r="C38">
         <v>18</v>
       </c>
       <c r="D38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" t="s">
         <v>87</v>
-      </c>
-      <c r="B39" t="s">
-        <v>88</v>
       </c>
       <c r="C39">
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>14</v>
+        <v>115</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>116</v>
       </c>
       <c r="C40">
-        <v>127</v>
+        <v>4</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
         <v>5</v>
       </c>
-      <c r="C41" t="s">
-        <v>63</v>
+      <c r="C41">
+        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B42" t="s">
-        <v>92</v>
-      </c>
-      <c r="C42">
-        <v>10</v>
-      </c>
-      <c r="D42" t="s">
-        <v>93</v>
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
-      </c>
-      <c r="C43" t="s">
-        <v>96</v>
+        <v>91</v>
+      </c>
+      <c r="C43">
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B44" t="s">
-        <v>99</v>
-      </c>
-      <c r="C44">
-        <v>20</v>
+        <v>94</v>
+      </c>
+      <c r="C44" t="s">
+        <v>95</v>
       </c>
       <c r="D44" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C45">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C46">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D46" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B47" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C47">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D47" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
-      </c>
-      <c r="C48" t="s">
-        <v>110</v>
+        <v>107</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>111</v>
+        <v>7</v>
       </c>
       <c r="B50" t="s">
-        <v>112</v>
+        <v>5</v>
       </c>
       <c r="C50" t="s">
-        <v>113</v>
+        <v>62</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>110</v>
+      </c>
+      <c r="B51" t="s">
         <v>111</v>
       </c>
-      <c r="B51" t="s">
-        <v>114</v>
-      </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>115</v>
+        <v>110</v>
+      </c>
+      <c r="B52" t="s">
+        <v>112</v>
+      </c>
+      <c r="C52" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D21" r:id="rId1" xr:uid="{7ACDA361-DC0B-4C1F-AD23-0AAD3D73CB22}"/>
+    <hyperlink ref="D23" r:id="rId2" xr:uid="{C988ED2F-D854-469D-A29A-C51F96CC8FBB}"/>
+    <hyperlink ref="D34" r:id="rId3" xr:uid="{95AF3F80-1357-49BF-8D66-CDDB0F3A24DD}"/>
+    <hyperlink ref="D31" r:id="rId4" xr:uid="{A906CE3A-D3EB-407B-9AB9-EF5F1802F1EA}"/>
+    <hyperlink ref="D9" r:id="rId5" xr:uid="{A4DDF58D-84B4-4D00-BC15-A2F288AFE0D5}"/>
+    <hyperlink ref="D16" r:id="rId6" xr:uid="{3B174B4A-90E7-472F-865E-4DF53409B68A}"/>
+    <hyperlink ref="D33" r:id="rId7" xr:uid="{FA59B98D-DF03-46B9-89F4-F08BBFD85B14}"/>
+    <hyperlink ref="D4" r:id="rId8" xr:uid="{CB4C4848-9775-4FE4-9978-57512BF0B79B}"/>
+    <hyperlink ref="D5" r:id="rId9" xr:uid="{9B5FA75F-B585-4B29-A4A7-7C498F3DD7B1}"/>
+    <hyperlink ref="D15" r:id="rId10" xr:uid="{2DC111E1-B766-4F6F-A625-E5E93B4A0015}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{21BDD5F9-9515-4746-8358-417654F6F39D}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{EF1FDAB3-81A8-4C4A-8FC1-16213CA7FAEE}"/>
+    <hyperlink ref="D25" r:id="rId13" xr:uid="{BAA439CB-3819-4C96-B8EE-4007E9D4CDF3}"/>
+    <hyperlink ref="D26" r:id="rId14" xr:uid="{45534430-F44A-4A4E-A33F-3CC05017C491}"/>
+    <hyperlink ref="D27" r:id="rId15" xr:uid="{E502074E-A16C-4D39-B708-4A9156300A54}"/>
+    <hyperlink ref="D40" r:id="rId16" xr:uid="{04D5E677-5A9A-4D09-AF28-567DC1E9408E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>